<commit_message>
add new column on inventaris ruangan
</commit_message>
<xml_diff>
--- a/public/template-inventaris-ruangan.xlsx
+++ b/public/template-inventaris-ruangan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24701"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\diakademik\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Digital Solusi Master\Diakad\diakademik\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1373E420-22EB-4016-8337-9817BFA15349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{599085F2-9FD0-48C1-AF05-2A1E6789CBC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{4063ED05-529A-4456-AE64-9D82F673D3C9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{4063ED05-529A-4456-AE64-9D82F673D3C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,19 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Nama Ruangan</t>
   </si>
@@ -74,6 +67,21 @@
   </si>
   <si>
     <t>DAPUR</t>
+  </si>
+  <si>
+    <t>Durasi Beli</t>
+  </si>
+  <si>
+    <t>Sumber Dana</t>
+  </si>
+  <si>
+    <t>Nama Vendor</t>
+  </si>
+  <si>
+    <t>Kas</t>
+  </si>
+  <si>
+    <t>Suya Elektronik</t>
   </si>
 </sst>
 </file>
@@ -137,7 +145,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -433,21 +441,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93881072-BE82-44D2-987F-EE94EE3E7FCA}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="16.44140625" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -461,22 +470,31 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -489,19 +507,28 @@
       <c r="D2" s="2">
         <v>44082</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="2">
+        <v>44082</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2">
         <v>10</v>
       </c>
-      <c r="F2">
+      <c r="I2">
         <v>10</v>
       </c>
-      <c r="G2">
+      <c r="J2">
         <v>0</v>
       </c>
-      <c r="H2" t="s">
+      <c r="K2" t="s">
         <v>11</v>
       </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>